<commit_message>
corrida 20260731 con Facts y defaulteados migrados
</commit_message>
<xml_diff>
--- a/01_INPUTS/MANUALES/REGLAS.xlsx
+++ b/01_INPUTS/MANUALES/REGLAS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="379">
   <si>
     <t>ID_Fund</t>
   </si>
@@ -505,6 +505,279 @@
   </si>
   <si>
     <t>Fecha_Fin</t>
+  </si>
+  <si>
+    <t>DEF</t>
+  </si>
+  <si>
+    <t>PROPDEF</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: ADASA 10% 07/30/2030 (fondos: ALTURAS II, MDLAT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CREDVA 8.875 02/07/2025 REGS (fondos: MCIT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: FOREBR 16 04/26/2028 INT 27012026 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: FOREBR 16 04/26/2028 INT 27042026 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: FOREBR 16 04/26/2028 INT 27102025 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: FOREBR 16 04/26/2028 INT 28072025 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GALLEO 13.75 03/04/2028 INT 04092025 (fondos: MCIT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GSHPBR 12 PERP 144A (fondos: MCIT, MLATHY)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LIGTBZ 0 08/31/2027 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: OIBRBZ 8.75 07/30/2026 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: SEAPT 16 01/29/2027 INT 29012026 (fondos: MCIT, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: SEAPT 16 01/29/27 INT 29012025 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: SEAPT 16 01/29/27 INT 29072025 (fondos: MCIT, MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIFIN 7 01/15/25 REGS (Escrow) CASH (fondos: MCIT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIFIN 7.375 02/12/26 REGS (Escrow) CASH (fondos: MCIT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIFIN 8.375 01/27/28 REGS (Escrow) CASH (fondos: MCIT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIGEL 13.5 12/31/2027 144A (fondos: MCIT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: BCOSAN 5.25 04/28/2005 (fondos: MDLAT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: BCOSAN 5.75 10/25/2005 EMTN (fondos: MDLAT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: BCOSAN 6 07/14/2005 EMTN (fondos: MDLAT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CASITA 7.5 06/29/2018 REGS (fondos: MDLAT)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CASITA F 06/28/2018 11 (fondos: MDLAT, MLCD, MLDL)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CIMTUP 8 12/07/2038 (fondos: MDLAT, MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GSHPBR 12 PERP Regs (fondos: MDLAT, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GOLITH 12 06/11/2020 (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GOLITH 15 06/11/2020 (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: INTSPN 0 PERP INTR (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: INTSPN 0 PERP INTr (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: INTSPN 0 PERP INtr (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: INTSPN 0 PERP Intr (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: INTSPN 7.5 01/24/2019 IN 241017 (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LN Converts (fondos: MLATHY, MLCD, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LN Participating Titles Part 1 (fondos: MLATHY, MLCD, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LN Participating Titles Part 2 (fondos: MLATHY, MLCD, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LUPABZ 0.4 PERP (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: OCEANO 11.25 07/15/2015 REGS (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: OCEANO 12 10/09/2018 (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: ORO SGP (fondos: MLATHY)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: OROSGP 12 12/20/2025 (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIFIN 7.25 09/27/23 REGS (Escrow) CASH (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIFIN 9.875 01/28/29 144A (Escrow) CASH (fondos: MLATHY, MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIGEL 13.5 12/31/2027 REGS (fondos: MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: UNIGNL 15 12/31/44 REGS (fondos: MLATHY, MLCC (Geneva), MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: BTOWBZ 8.35 07/26/2029 G2 (fondos: MLCC (Geneva))</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CASITA 7.5 06/29/2018 144A (fondos: MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CREAL 8 01/21/2028 REGS - Escrow (fondos: MLCD)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: APICBZ 3.602 07/16/2029 26 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: APICBZ 6.0081 10/15/2030 73-1 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: APICBZ 6.2513 10/17/2033 73-2 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: APICBZ 6.5885 08/16/2032 38-1 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: APICBZ 6.7382 08/17/2037 38-2 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: BRASKM F 11/09/2029 A81 (fondos: MLDL)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 3.539 11/15/2029 14 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 5.8 06/15/2030 15 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 5.9219 03/15/2029 17 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 5.9645 03/15/2032 27 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 6.4794 09/15/2039 23 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ 6.4879 09/15/2034 13 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RAIZBZ Float 07/15/2030 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: RBCSBZ 4.04 03/16/2026 2-2 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 2.875 04/22/2028 19-B (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 3.09375 05/15/2030 A (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 3.125 05/22/2028 37-B (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 3.625 07/13/2027 19-A (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 5.5 04/19/2025 A (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFB 7.28125 10/16/2026 (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: TELEFO 7.375 04/10/2027 REGS (fondos: MLDL, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: ELFABZ Float 04/13/2028 (fondos: MLDL)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PCARBZ F 05/10/2028 B8 (fondos: MLDL)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LC PAG PUERTO VARAS 6.60% 31012028 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: LC QUINTERO ENERGIA 1,00% 15/01/2028 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG ARAUCO ARJ 3.00 30/06/2025 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG ARAUCO ARJ 3.00 30/12/2027 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG ARAUCO CONC 7.47 30/06/2021 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 08/08/2023 - C DESM I B (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 08/08/2023 - C DESM II A (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 08/08/2023 - C DESM III (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 30/06/2021 - B DESM I (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 30/06/2021 - B DESM II (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 30/06/2021 - B DESM III (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 12% 30/06/2021 - B DESM III - II (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: PAG MICROBLEND 6% 08/08/2023 - A (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: ENJOY 8 07/10/2029 A (fondos: MDCH, MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: GFMEGA 8.25 02/11/2025 REGS (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CZRSBZ 7 07/08/2013 1 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CZRSBZ 7.625 04/21/2014 (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CZRSBZ 8 09/17/2012 EMTN (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CZRSBZ 8.25 01/20/2016 REGS (fondos: MRCLP)</t>
+  </si>
+  <si>
+    <t>migrado de DEFAULTEADOS.xlsx: CZRSBZ 8.5 02/20/2015 REGS (fondos: MRCLP)</t>
   </si>
   <si>
     <t>SubID_Instrumento</t>
@@ -2630,7 +2903,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2651,6 +2924,985 @@
       </c>
       <c r="F1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="B2">
+        <v>441</v>
+      </c>
+      <c r="C2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="B3">
+        <v>4286</v>
+      </c>
+      <c r="C3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="B4">
+        <v>204645</v>
+      </c>
+      <c r="C4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="B5">
+        <v>214791</v>
+      </c>
+      <c r="C5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="B6">
+        <v>193873</v>
+      </c>
+      <c r="C6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="B7">
+        <v>181402</v>
+      </c>
+      <c r="C7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="B8">
+        <v>199992</v>
+      </c>
+      <c r="C8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="B9">
+        <v>151465</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+      <c r="F9" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="B10">
+        <v>159173</v>
+      </c>
+      <c r="C10" t="s">
+        <v>162</v>
+      </c>
+      <c r="F10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="B11">
+        <v>32259</v>
+      </c>
+      <c r="C11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="B12">
+        <v>205354</v>
+      </c>
+      <c r="C12" t="s">
+        <v>161</v>
+      </c>
+      <c r="F12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="B13">
+        <v>161099</v>
+      </c>
+      <c r="C13" t="s">
+        <v>161</v>
+      </c>
+      <c r="F13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="B14">
+        <v>181048</v>
+      </c>
+      <c r="C14" t="s">
+        <v>161</v>
+      </c>
+      <c r="F14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="B15">
+        <v>135285</v>
+      </c>
+      <c r="C15" t="s">
+        <v>162</v>
+      </c>
+      <c r="F15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="B16">
+        <v>135282</v>
+      </c>
+      <c r="C16" t="s">
+        <v>162</v>
+      </c>
+      <c r="F16" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="B17">
+        <v>135280</v>
+      </c>
+      <c r="C17" t="s">
+        <v>162</v>
+      </c>
+      <c r="F17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18">
+        <v>161090</v>
+      </c>
+      <c r="C18" t="s">
+        <v>161</v>
+      </c>
+      <c r="F18" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19">
+        <v>583</v>
+      </c>
+      <c r="C19" t="s">
+        <v>161</v>
+      </c>
+      <c r="F19" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20">
+        <v>584</v>
+      </c>
+      <c r="C20" t="s">
+        <v>161</v>
+      </c>
+      <c r="F20" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21">
+        <v>585</v>
+      </c>
+      <c r="C21" t="s">
+        <v>161</v>
+      </c>
+      <c r="F21" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22">
+        <v>715</v>
+      </c>
+      <c r="C22" t="s">
+        <v>161</v>
+      </c>
+      <c r="F22" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23">
+        <v>716</v>
+      </c>
+      <c r="C23" t="s">
+        <v>161</v>
+      </c>
+      <c r="F23" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24">
+        <v>157263</v>
+      </c>
+      <c r="C24" t="s">
+        <v>161</v>
+      </c>
+      <c r="F24" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="B25">
+        <v>849</v>
+      </c>
+      <c r="C25" t="s">
+        <v>162</v>
+      </c>
+      <c r="F25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="B26">
+        <v>840</v>
+      </c>
+      <c r="C26" t="s">
+        <v>162</v>
+      </c>
+      <c r="F26" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="B27">
+        <v>841</v>
+      </c>
+      <c r="C27" t="s">
+        <v>162</v>
+      </c>
+      <c r="F27" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="B28">
+        <v>31128</v>
+      </c>
+      <c r="C28" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="B29">
+        <v>31129</v>
+      </c>
+      <c r="C29" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="B30">
+        <v>31130</v>
+      </c>
+      <c r="C30" t="s">
+        <v>161</v>
+      </c>
+      <c r="F30" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="B31">
+        <v>31131</v>
+      </c>
+      <c r="C31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6">
+      <c r="B32">
+        <v>865</v>
+      </c>
+      <c r="C32" t="s">
+        <v>161</v>
+      </c>
+      <c r="F32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33">
+        <v>213458</v>
+      </c>
+      <c r="C33" t="s">
+        <v>162</v>
+      </c>
+      <c r="F33" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6">
+      <c r="B34">
+        <v>213459</v>
+      </c>
+      <c r="C34" t="s">
+        <v>162</v>
+      </c>
+      <c r="F34" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6">
+      <c r="B35">
+        <v>213460</v>
+      </c>
+      <c r="C35" t="s">
+        <v>162</v>
+      </c>
+      <c r="F35" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
+      <c r="B36">
+        <v>35811</v>
+      </c>
+      <c r="C36" t="s">
+        <v>161</v>
+      </c>
+      <c r="F36" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6">
+      <c r="B37">
+        <v>928</v>
+      </c>
+      <c r="C37" t="s">
+        <v>161</v>
+      </c>
+      <c r="F37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6">
+      <c r="B38">
+        <v>929</v>
+      </c>
+      <c r="C38" t="s">
+        <v>161</v>
+      </c>
+      <c r="F38" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6">
+      <c r="B39">
+        <v>219502</v>
+      </c>
+      <c r="C39" t="s">
+        <v>162</v>
+      </c>
+      <c r="F39" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6">
+      <c r="B40">
+        <v>941</v>
+      </c>
+      <c r="C40" t="s">
+        <v>161</v>
+      </c>
+      <c r="F40" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6">
+      <c r="B41">
+        <v>135284</v>
+      </c>
+      <c r="C41" t="s">
+        <v>162</v>
+      </c>
+      <c r="F41" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6">
+      <c r="B42">
+        <v>135286</v>
+      </c>
+      <c r="C42" t="s">
+        <v>162</v>
+      </c>
+      <c r="F42" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6">
+      <c r="B43">
+        <v>161091</v>
+      </c>
+      <c r="C43" t="s">
+        <v>161</v>
+      </c>
+      <c r="F43" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6">
+      <c r="B44">
+        <v>161001</v>
+      </c>
+      <c r="C44" t="s">
+        <v>161</v>
+      </c>
+      <c r="F44" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6">
+      <c r="B45">
+        <v>201208</v>
+      </c>
+      <c r="C45" t="s">
+        <v>162</v>
+      </c>
+      <c r="F45" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6">
+      <c r="B46">
+        <v>714</v>
+      </c>
+      <c r="C46" t="s">
+        <v>161</v>
+      </c>
+      <c r="F46" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6">
+      <c r="B47">
+        <v>171365</v>
+      </c>
+      <c r="C47" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6">
+      <c r="B48">
+        <v>209439</v>
+      </c>
+      <c r="C48" t="s">
+        <v>161</v>
+      </c>
+      <c r="F48" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6">
+      <c r="B49">
+        <v>209273</v>
+      </c>
+      <c r="C49" t="s">
+        <v>161</v>
+      </c>
+      <c r="F49" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6">
+      <c r="B50">
+        <v>226683</v>
+      </c>
+      <c r="C50" t="s">
+        <v>161</v>
+      </c>
+      <c r="F50" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6">
+      <c r="B51">
+        <v>226684</v>
+      </c>
+      <c r="C51" t="s">
+        <v>161</v>
+      </c>
+      <c r="F51" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6">
+      <c r="B52">
+        <v>226685</v>
+      </c>
+      <c r="C52" t="s">
+        <v>161</v>
+      </c>
+      <c r="F52" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6">
+      <c r="B53">
+        <v>115460</v>
+      </c>
+      <c r="C53" t="s">
+        <v>161</v>
+      </c>
+      <c r="F53" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6">
+      <c r="B54">
+        <v>205494</v>
+      </c>
+      <c r="C54" t="s">
+        <v>161</v>
+      </c>
+      <c r="F54" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6">
+      <c r="B55">
+        <v>226885</v>
+      </c>
+      <c r="C55" t="s">
+        <v>161</v>
+      </c>
+      <c r="F55" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6">
+      <c r="B56">
+        <v>222699</v>
+      </c>
+      <c r="C56" t="s">
+        <v>161</v>
+      </c>
+      <c r="F56" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6">
+      <c r="B57">
+        <v>226996</v>
+      </c>
+      <c r="C57" t="s">
+        <v>161</v>
+      </c>
+      <c r="F57" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6">
+      <c r="B58">
+        <v>227576</v>
+      </c>
+      <c r="C58" t="s">
+        <v>161</v>
+      </c>
+      <c r="F58" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6">
+      <c r="B59">
+        <v>203106</v>
+      </c>
+      <c r="C59" t="s">
+        <v>161</v>
+      </c>
+      <c r="F59" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6">
+      <c r="B60">
+        <v>208992</v>
+      </c>
+      <c r="C60" t="s">
+        <v>161</v>
+      </c>
+      <c r="F60" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6">
+      <c r="B61">
+        <v>226886</v>
+      </c>
+      <c r="C61" t="s">
+        <v>161</v>
+      </c>
+      <c r="F61" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6">
+      <c r="B62">
+        <v>175782</v>
+      </c>
+      <c r="C62" t="s">
+        <v>161</v>
+      </c>
+      <c r="F62" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6">
+      <c r="B63">
+        <v>176588</v>
+      </c>
+      <c r="C63" t="s">
+        <v>161</v>
+      </c>
+      <c r="F63" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6">
+      <c r="B64">
+        <v>175802</v>
+      </c>
+      <c r="C64" t="s">
+        <v>161</v>
+      </c>
+      <c r="F64" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6">
+      <c r="B65">
+        <v>175703</v>
+      </c>
+      <c r="C65" t="s">
+        <v>161</v>
+      </c>
+      <c r="F65" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6">
+      <c r="B66">
+        <v>173738</v>
+      </c>
+      <c r="C66" t="s">
+        <v>161</v>
+      </c>
+      <c r="F66" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6">
+      <c r="B67">
+        <v>175702</v>
+      </c>
+      <c r="C67" t="s">
+        <v>161</v>
+      </c>
+      <c r="F67" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6">
+      <c r="B68">
+        <v>1090</v>
+      </c>
+      <c r="C68" t="s">
+        <v>161</v>
+      </c>
+      <c r="F68" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6">
+      <c r="B69">
+        <v>115862</v>
+      </c>
+      <c r="C69" t="s">
+        <v>162</v>
+      </c>
+      <c r="F69" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6">
+      <c r="B70">
+        <v>130023</v>
+      </c>
+      <c r="C70" t="s">
+        <v>162</v>
+      </c>
+      <c r="F70" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6">
+      <c r="B71">
+        <v>205779</v>
+      </c>
+      <c r="C71" t="s">
+        <v>161</v>
+      </c>
+      <c r="F71" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6">
+      <c r="B72">
+        <v>160240</v>
+      </c>
+      <c r="C72" t="s">
+        <v>161</v>
+      </c>
+      <c r="F72" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6">
+      <c r="B73">
+        <v>31509</v>
+      </c>
+      <c r="C73" t="s">
+        <v>161</v>
+      </c>
+      <c r="F73" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6">
+      <c r="B74">
+        <v>31510</v>
+      </c>
+      <c r="C74" t="s">
+        <v>161</v>
+      </c>
+      <c r="F74" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6">
+      <c r="B75">
+        <v>3334</v>
+      </c>
+      <c r="C75" t="s">
+        <v>161</v>
+      </c>
+      <c r="F75" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6">
+      <c r="B76">
+        <v>31179</v>
+      </c>
+      <c r="C76" t="s">
+        <v>161</v>
+      </c>
+      <c r="F76" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6">
+      <c r="B77">
+        <v>3946</v>
+      </c>
+      <c r="C77" t="s">
+        <v>161</v>
+      </c>
+      <c r="F77" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6">
+      <c r="B78">
+        <v>3947</v>
+      </c>
+      <c r="C78" t="s">
+        <v>161</v>
+      </c>
+      <c r="F78" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6">
+      <c r="B79">
+        <v>3948</v>
+      </c>
+      <c r="C79" t="s">
+        <v>161</v>
+      </c>
+      <c r="F79" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6">
+      <c r="B80">
+        <v>3949</v>
+      </c>
+      <c r="C80" t="s">
+        <v>161</v>
+      </c>
+      <c r="F80" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6">
+      <c r="B81">
+        <v>3950</v>
+      </c>
+      <c r="C81" t="s">
+        <v>161</v>
+      </c>
+      <c r="F81" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6">
+      <c r="B82">
+        <v>31600</v>
+      </c>
+      <c r="C82" t="s">
+        <v>161</v>
+      </c>
+      <c r="F82" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6">
+      <c r="B83">
+        <v>3951</v>
+      </c>
+      <c r="C83" t="s">
+        <v>161</v>
+      </c>
+      <c r="F83" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6">
+      <c r="B84">
+        <v>160766</v>
+      </c>
+      <c r="C84" t="s">
+        <v>161</v>
+      </c>
+      <c r="F84" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6">
+      <c r="B85">
+        <v>4311</v>
+      </c>
+      <c r="C85" t="s">
+        <v>161</v>
+      </c>
+      <c r="F85" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6">
+      <c r="B86">
+        <v>771</v>
+      </c>
+      <c r="C86" t="s">
+        <v>161</v>
+      </c>
+      <c r="F86" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6">
+      <c r="B87">
+        <v>772</v>
+      </c>
+      <c r="C87" t="s">
+        <v>161</v>
+      </c>
+      <c r="F87" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6">
+      <c r="B88">
+        <v>773</v>
+      </c>
+      <c r="C88" t="s">
+        <v>161</v>
+      </c>
+      <c r="F88" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6">
+      <c r="B89">
+        <v>775</v>
+      </c>
+      <c r="C89" t="s">
+        <v>161</v>
+      </c>
+      <c r="F89" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6">
+      <c r="B90">
+        <v>777</v>
+      </c>
+      <c r="C90" t="s">
+        <v>161</v>
+      </c>
+      <c r="F90" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -2671,13 +3923,13 @@
         <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>161</v>
+        <v>252</v>
       </c>
       <c r="D1" t="s">
-        <v>162</v>
+        <v>253</v>
       </c>
       <c r="E1" t="s">
-        <v>163</v>
+        <v>254</v>
       </c>
       <c r="F1" t="s">
         <v>159</v>
@@ -2686,7 +3938,7 @@
         <v>160</v>
       </c>
       <c r="H1" t="s">
-        <v>164</v>
+        <v>255</v>
       </c>
       <c r="I1" t="s">
         <v>2</v>
@@ -2710,13 +3962,13 @@
         <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>161</v>
+        <v>252</v>
       </c>
       <c r="D1" t="s">
-        <v>165</v>
+        <v>256</v>
       </c>
       <c r="E1" t="s">
-        <v>166</v>
+        <v>257</v>
       </c>
       <c r="F1" t="s">
         <v>159</v>
@@ -2739,13 +3991,13 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E2" t="s">
-        <v>168</v>
+        <v>259</v>
       </c>
       <c r="H2" t="s">
-        <v>176</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2759,13 +4011,13 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E3" t="s">
-        <v>169</v>
+        <v>260</v>
       </c>
       <c r="H3" t="s">
-        <v>177</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2779,13 +4031,13 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E4" t="s">
-        <v>169</v>
+        <v>260</v>
       </c>
       <c r="H4" t="s">
-        <v>178</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2799,13 +4051,13 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E5" t="s">
-        <v>169</v>
+        <v>260</v>
       </c>
       <c r="H5" t="s">
-        <v>179</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2819,13 +4071,13 @@
         <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E6" t="s">
-        <v>170</v>
+        <v>261</v>
       </c>
       <c r="H6" t="s">
-        <v>180</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2839,13 +4091,13 @@
         <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E7" t="s">
-        <v>171</v>
+        <v>262</v>
       </c>
       <c r="H7" t="s">
-        <v>181</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2859,13 +4111,13 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E8" t="s">
-        <v>170</v>
+        <v>261</v>
       </c>
       <c r="H8" t="s">
-        <v>182</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2879,13 +4131,13 @@
         <v>196</v>
       </c>
       <c r="D9" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E9" t="s">
-        <v>168</v>
+        <v>259</v>
       </c>
       <c r="H9" t="s">
-        <v>183</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2899,13 +4151,13 @@
         <v>123</v>
       </c>
       <c r="D10" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E10" t="s">
-        <v>172</v>
+        <v>263</v>
       </c>
       <c r="H10" t="s">
-        <v>184</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2919,13 +4171,13 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E11" t="s">
-        <v>173</v>
+        <v>264</v>
       </c>
       <c r="H11" t="s">
-        <v>185</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2939,13 +4191,13 @@
         <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E12" t="s">
-        <v>174</v>
+        <v>265</v>
       </c>
       <c r="H12" t="s">
-        <v>186</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2959,13 +4211,13 @@
         <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E13" t="s">
-        <v>175</v>
+        <v>266</v>
       </c>
       <c r="H13" t="s">
-        <v>187</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2979,13 +4231,13 @@
         <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="E14" t="s">
-        <v>175</v>
+        <v>266</v>
       </c>
       <c r="H14" t="s">
-        <v>188</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -3003,452 +4255,452 @@
         <v>29</v>
       </c>
       <c r="B1" t="s">
-        <v>189</v>
+        <v>280</v>
       </c>
       <c r="C1" t="s">
-        <v>190</v>
+        <v>281</v>
       </c>
       <c r="D1" t="s">
-        <v>191</v>
+        <v>282</v>
       </c>
       <c r="E1" t="s">
-        <v>192</v>
+        <v>283</v>
       </c>
       <c r="F1" t="s">
-        <v>193</v>
+        <v>284</v>
       </c>
       <c r="G1" t="s">
         <v>0</v>
       </c>
       <c r="H1" t="s">
-        <v>194</v>
+        <v>285</v>
       </c>
       <c r="I1" t="s">
-        <v>195</v>
+        <v>286</v>
       </c>
       <c r="J1" t="s">
-        <v>196</v>
+        <v>287</v>
       </c>
       <c r="K1" t="s">
-        <v>197</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>289</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>302</v>
       </c>
       <c r="C2" t="s">
-        <v>162</v>
+        <v>253</v>
       </c>
       <c r="D2" t="s">
-        <v>232</v>
+        <v>323</v>
       </c>
       <c r="E2" t="s">
-        <v>238</v>
+        <v>329</v>
       </c>
       <c r="F2" t="s">
-        <v>244</v>
+        <v>335</v>
       </c>
       <c r="H2" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I2" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J2" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K2" t="s">
-        <v>252</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>198</v>
+        <v>289</v>
       </c>
       <c r="B3" t="s">
-        <v>211</v>
+        <v>302</v>
       </c>
       <c r="C3" t="s">
-        <v>162</v>
+        <v>253</v>
       </c>
       <c r="D3" t="s">
-        <v>232</v>
+        <v>323</v>
       </c>
       <c r="E3" t="s">
-        <v>239</v>
+        <v>330</v>
       </c>
       <c r="F3" t="s">
-        <v>244</v>
+        <v>335</v>
       </c>
       <c r="G3">
         <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I3" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J3" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K3" t="s">
-        <v>253</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>199</v>
+        <v>290</v>
       </c>
       <c r="B4" t="s">
-        <v>212</v>
+        <v>303</v>
       </c>
       <c r="C4" t="s">
-        <v>162</v>
+        <v>253</v>
       </c>
       <c r="D4" t="s">
-        <v>233</v>
+        <v>324</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>245</v>
+        <v>336</v>
       </c>
       <c r="H4" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I4" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J4" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K4" t="s">
-        <v>254</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>200</v>
+        <v>291</v>
       </c>
       <c r="B5" t="s">
-        <v>213</v>
+        <v>304</v>
       </c>
       <c r="C5" t="s">
-        <v>224</v>
+        <v>315</v>
       </c>
       <c r="D5" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="F5" t="s">
-        <v>245</v>
+        <v>336</v>
       </c>
       <c r="H5" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I5" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J5" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K5" t="s">
-        <v>255</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>305</v>
       </c>
       <c r="C6" t="s">
-        <v>225</v>
+        <v>316</v>
       </c>
       <c r="D6" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="F6" t="s">
-        <v>246</v>
+        <v>337</v>
       </c>
       <c r="H6" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I6" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J6" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K6" t="s">
-        <v>256</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>293</v>
       </c>
       <c r="B7" t="s">
-        <v>215</v>
+        <v>306</v>
       </c>
       <c r="C7" t="s">
-        <v>226</v>
+        <v>317</v>
       </c>
       <c r="D7" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="F7" t="s">
-        <v>244</v>
+        <v>335</v>
       </c>
       <c r="H7" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I7" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="J7" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K7" t="s">
-        <v>257</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>294</v>
       </c>
       <c r="B8" t="s">
-        <v>216</v>
+        <v>307</v>
       </c>
       <c r="C8" t="s">
-        <v>227</v>
+        <v>318</v>
       </c>
       <c r="D8" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="F8" t="s">
-        <v>246</v>
+        <v>337</v>
       </c>
       <c r="H8" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I8" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="J8" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K8" t="s">
-        <v>258</v>
+        <v>349</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>204</v>
+        <v>295</v>
       </c>
       <c r="B9" t="s">
-        <v>217</v>
+        <v>308</v>
       </c>
       <c r="C9" t="s">
-        <v>228</v>
+        <v>319</v>
       </c>
       <c r="D9" t="s">
-        <v>235</v>
+        <v>326</v>
       </c>
       <c r="E9" t="s">
-        <v>240</v>
+        <v>331</v>
       </c>
       <c r="F9" t="s">
-        <v>245</v>
+        <v>336</v>
       </c>
       <c r="H9" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I9" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="J9" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K9" t="s">
-        <v>259</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>296</v>
       </c>
       <c r="B10" t="s">
-        <v>218</v>
+        <v>309</v>
       </c>
       <c r="C10" t="s">
-        <v>229</v>
+        <v>320</v>
       </c>
       <c r="D10" t="s">
-        <v>233</v>
+        <v>324</v>
       </c>
       <c r="E10" t="s">
-        <v>241</v>
+        <v>332</v>
       </c>
       <c r="F10" t="s">
-        <v>245</v>
+        <v>336</v>
       </c>
       <c r="H10" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I10" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J10" t="s">
-        <v>251</v>
+        <v>342</v>
       </c>
       <c r="K10" t="s">
-        <v>260</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>297</v>
       </c>
       <c r="B11" t="s">
-        <v>219</v>
+        <v>310</v>
       </c>
       <c r="C11" t="s">
-        <v>230</v>
+        <v>321</v>
       </c>
       <c r="D11" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="F11" t="s">
-        <v>245</v>
+        <v>336</v>
       </c>
       <c r="H11" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="I11" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J11" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K11" t="s">
-        <v>261</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>207</v>
+        <v>298</v>
       </c>
       <c r="B12" t="s">
-        <v>220</v>
+        <v>311</v>
       </c>
       <c r="C12" t="s">
-        <v>231</v>
+        <v>322</v>
       </c>
       <c r="D12" t="s">
-        <v>236</v>
+        <v>327</v>
       </c>
       <c r="E12" t="s">
-        <v>242</v>
+        <v>333</v>
       </c>
       <c r="F12" t="s">
-        <v>247</v>
+        <v>338</v>
       </c>
       <c r="H12" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="I12" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J12" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K12" t="s">
-        <v>262</v>
+        <v>353</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>208</v>
+        <v>299</v>
       </c>
       <c r="B13" t="s">
-        <v>221</v>
+        <v>312</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>237</v>
+        <v>328</v>
       </c>
       <c r="E13" t="s">
-        <v>243</v>
+        <v>334</v>
       </c>
       <c r="F13" t="s">
-        <v>247</v>
+        <v>338</v>
       </c>
       <c r="H13" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="I13" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J13" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K13" t="s">
-        <v>263</v>
+        <v>354</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>209</v>
+        <v>300</v>
       </c>
       <c r="B14" t="s">
-        <v>222</v>
+        <v>313</v>
       </c>
       <c r="F14" t="s">
-        <v>246</v>
+        <v>337</v>
       </c>
       <c r="H14" t="s">
-        <v>248</v>
+        <v>339</v>
       </c>
       <c r="I14" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J14" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K14" t="s">
-        <v>264</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>210</v>
+        <v>301</v>
       </c>
       <c r="B15" t="s">
-        <v>223</v>
+        <v>314</v>
       </c>
       <c r="F15" t="s">
-        <v>247</v>
+        <v>338</v>
       </c>
       <c r="H15" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="I15" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="J15" t="s">
-        <v>250</v>
+        <v>341</v>
       </c>
       <c r="K15" t="s">
-        <v>265</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -3463,123 +4715,123 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>266</v>
+        <v>357</v>
       </c>
       <c r="B1" t="s">
         <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>267</v>
+        <v>358</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>278</v>
+        <v>369</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>268</v>
+        <v>359</v>
       </c>
       <c r="B3">
         <v>-0.5</v>
       </c>
       <c r="C3" t="s">
-        <v>279</v>
+        <v>370</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>269</v>
+        <v>360</v>
       </c>
       <c r="B4">
         <v>0.01</v>
       </c>
       <c r="C4" t="s">
-        <v>280</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>270</v>
+        <v>361</v>
       </c>
       <c r="B5">
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>281</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>271</v>
+        <v>362</v>
       </c>
       <c r="B6" t="s">
-        <v>277</v>
+        <v>368</v>
       </c>
       <c r="C6" t="s">
-        <v>282</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>272</v>
+        <v>363</v>
       </c>
       <c r="B7">
         <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>283</v>
+        <v>374</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>273</v>
+        <v>364</v>
       </c>
       <c r="B8">
         <v>0.25</v>
       </c>
       <c r="C8" t="s">
-        <v>284</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>274</v>
+        <v>365</v>
       </c>
       <c r="B9">
         <v>0.4</v>
       </c>
       <c r="C9" t="s">
-        <v>285</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>275</v>
+        <v>366</v>
       </c>
       <c r="B10">
         <v>0.1</v>
       </c>
       <c r="C10" t="s">
-        <v>286</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>276</v>
+        <v>367</v>
       </c>
       <c r="B11">
         <v>0.95</v>
       </c>
       <c r="C11" t="s">
-        <v>287</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
REGLAS sin filas BalSheetKey
</commit_message>
<xml_diff>
--- a/01_INPUTS/MANUALES/REGLAS.xlsx
+++ b/01_INPUTS/MANUALES/REGLAS.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Moneda03\Compartidos\Inteligencia de Negocios y Mercados\Desarrollo\Cristopher Olmedo\Reporteria 2.0\01_INPUTS\MANUALES\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99EB12DB-7FF2-45DB-8974-CF65BFA89EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-28920" yWindow="1635" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fondos" sheetId="1" r:id="rId1"/>
@@ -17,12 +23,25 @@
     <sheet name="alertas" sheetId="8" r:id="rId8"/>
     <sheet name="parametros" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="368">
   <si>
     <t>ID_Fund</t>
   </si>
@@ -120,30 +139,12 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>BalSheetKey</t>
-  </si>
-  <si>
     <t>PK2</t>
   </si>
   <si>
     <t>Issue_Type_Code</t>
   </si>
   <si>
-    <t>Asset11412000</t>
-  </si>
-  <si>
-    <t>Asset11432000</t>
-  </si>
-  <si>
-    <t>Asset12422000</t>
-  </si>
-  <si>
-    <t>Asset12812000</t>
-  </si>
-  <si>
-    <t>Asset12832000</t>
-  </si>
-  <si>
     <t>176142-38</t>
   </si>
   <si>
@@ -151,21 +152,6 @@
   </si>
   <si>
     <t>FACTURA</t>
-  </si>
-  <si>
-    <t>MRCLP: depósito fijo (Issue 4) es caja</t>
-  </si>
-  <si>
-    <t>MRCLP: depósito inflation-linked es caja</t>
-  </si>
-  <si>
-    <t>MRCLP: depósito soberano flotante es caja</t>
-  </si>
-  <si>
-    <t>MRCLP: pagaré soberano fijo es caja</t>
-  </si>
-  <si>
-    <t>MRCLP: pagaré soberano inflation-linked es caja</t>
   </si>
   <si>
     <t>FIP ALZA RENTAS COMERCIALES II — Treatment Equity</t>
@@ -1164,8 +1150,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1202,13 +1188,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1246,7 +1240,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1280,6 +1274,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1314,9 +1309,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1489,11 +1485,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="45.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1504,7 +1503,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>11</v>
       </c>
@@ -1515,7 +1514,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>20</v>
       </c>
@@ -1526,7 +1525,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>17</v>
       </c>
@@ -1543,11 +1542,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1558,7 +1561,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1569,7 +1572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1580,7 +1583,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1591,7 +1594,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1602,7 +1605,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1613,7 +1616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1624,7 +1627,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1635,7 +1638,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1646,7 +1649,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1668,7 +1671,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1679,7 +1682,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1690,7 +1693,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1701,7 +1704,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1712,7 +1715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1729,11 +1732,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="62.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -1756,7 +1768,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1767,130 +1779,30 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>20</v>
-      </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
         <v>36</v>
       </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
       <c r="G3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
         <v>38</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1899,61 +1811,69 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F69"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="62.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D4">
         <v>-0.02</v>
@@ -1962,144 +1882,144 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D5">
-        <v>0.0429</v>
+        <v>4.2900000000000001E-2</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>65</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D7">
-        <v>0.0465</v>
+        <v>4.65E-2</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>65</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="F10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="F11" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F12" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D13">
-        <v>-0.0012</v>
+        <v>-1.1999999999999999E-3</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D14">
         <v>-0.01</v>
@@ -2108,18 +2028,18 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D15">
         <v>-0.02</v>
@@ -2128,18 +2048,18 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D16">
         <v>-0.02</v>
@@ -2148,58 +2068,58 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D17">
-        <v>0.0429</v>
+        <v>4.2900000000000001E-2</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D18">
-        <v>0.082</v>
+        <v>8.2000000000000003E-2</v>
       </c>
       <c r="E18">
         <v>1377</v>
       </c>
       <c r="F18" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>59</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D19">
         <v>-0.02</v>
@@ -2208,18 +2128,18 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D20">
         <v>-0.02</v>
@@ -2228,18 +2148,18 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D21">
         <v>-0.02</v>
@@ -2248,18 +2168,18 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -2268,18 +2188,18 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D23">
         <v>-0.02</v>
@@ -2288,18 +2208,18 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D24">
         <v>-0.02</v>
@@ -2308,38 +2228,38 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>59</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D25">
-        <v>0.0429</v>
+        <v>4.2900000000000001E-2</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C26" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D26">
         <v>-0.02</v>
@@ -2348,29 +2268,29 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="F27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -2379,18 +2299,18 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D29">
         <v>-0.02</v>
@@ -2399,18 +2319,18 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C30" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D30">
         <v>-0.02</v>
@@ -2419,40 +2339,40 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="F32" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="D33">
         <v>-0.02</v>
@@ -2461,38 +2381,38 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C34" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D34">
-        <v>0.016</v>
+        <v>1.6E-2</v>
       </c>
       <c r="E34">
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D35">
         <v>-0.02</v>
@@ -2501,51 +2421,51 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="F36" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="F37" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="F38" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="C39" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D39">
         <v>-0.02</v>
@@ -2554,18 +2474,18 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C40" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D40">
         <v>-0.02</v>
@@ -2574,326 +2494,326 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>16</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>17</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F42" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F43" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F44" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F45" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F46" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F47" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="F48" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>17</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="F49" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>17</v>
       </c>
       <c r="B50" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="F50" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>17</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="F51" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>17</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="F52" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>17</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="F53" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>17</v>
       </c>
       <c r="B54" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F54" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>17</v>
       </c>
       <c r="B55" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="F55" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>17</v>
       </c>
       <c r="B56" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="F56" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>17</v>
       </c>
       <c r="B57" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="F57" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>17</v>
       </c>
       <c r="B58" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F58" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>17</v>
       </c>
       <c r="B59" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F59" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>17</v>
       </c>
       <c r="B60" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="F60" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>17</v>
       </c>
       <c r="B61" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="F61" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>17</v>
       </c>
       <c r="B62" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="F62" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>17</v>
       </c>
       <c r="B63" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="F63" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>17</v>
       </c>
       <c r="B64" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="F64" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>17</v>
       </c>
       <c r="B65" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="F65" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>17</v>
       </c>
       <c r="B66" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="F66" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>17</v>
       </c>
       <c r="B67" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="F67" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>17</v>
       </c>
       <c r="B68" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="F68" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>17</v>
       </c>
       <c r="B69" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F69" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2902,1007 +2822,1011 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F90"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C1" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D1" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E1" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>441</v>
       </c>
       <c r="C2" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>4286</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F3" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>204645</v>
       </c>
       <c r="C4" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>214791</v>
       </c>
       <c r="C5" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>193873</v>
       </c>
       <c r="C6" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F6" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>181402</v>
       </c>
       <c r="C7" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F7" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>199992</v>
       </c>
       <c r="C8" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F8" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>151465</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F9" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>159173</v>
       </c>
       <c r="C10" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>32259</v>
       </c>
       <c r="C11" t="s">
+        <v>150</v>
+      </c>
+      <c r="F11" t="s">
         <v>161</v>
       </c>
-      <c r="F11" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>205354</v>
       </c>
       <c r="C12" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F12" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>161099</v>
       </c>
       <c r="C13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>181048</v>
       </c>
       <c r="C14" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F14" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>135285</v>
       </c>
       <c r="C15" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F15" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>135282</v>
       </c>
       <c r="C16" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F16" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>135280</v>
       </c>
       <c r="C17" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F17" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>161090</v>
       </c>
       <c r="C18" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F18" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>583</v>
       </c>
       <c r="C19" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F19" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>584</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F20" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>585</v>
       </c>
       <c r="C21" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>715</v>
       </c>
       <c r="C22" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F22" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>716</v>
       </c>
       <c r="C23" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F23" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>157263</v>
       </c>
       <c r="C24" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F24" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>849</v>
       </c>
       <c r="C25" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F25" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>840</v>
       </c>
       <c r="C26" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F26" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>841</v>
       </c>
       <c r="C27" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F27" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>31128</v>
       </c>
       <c r="C28" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F28" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>31129</v>
       </c>
       <c r="C29" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F29" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>31130</v>
       </c>
       <c r="C30" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F30" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>31131</v>
       </c>
       <c r="C31" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F31" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32">
         <v>865</v>
       </c>
       <c r="C32" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F32" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>213458</v>
       </c>
       <c r="C33" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F33" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>213459</v>
       </c>
       <c r="C34" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F34" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>213460</v>
       </c>
       <c r="C35" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F35" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>35811</v>
       </c>
       <c r="C36" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F36" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37">
         <v>928</v>
       </c>
       <c r="C37" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F37" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38">
         <v>929</v>
       </c>
       <c r="C38" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F38" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39">
         <v>219502</v>
       </c>
       <c r="C39" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F39" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40">
         <v>941</v>
       </c>
       <c r="C40" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F40" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41">
         <v>135284</v>
       </c>
       <c r="C41" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F41" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42">
         <v>135286</v>
       </c>
       <c r="C42" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F42" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43">
         <v>161091</v>
       </c>
       <c r="C43" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F43" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44">
         <v>161001</v>
       </c>
       <c r="C44" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F44" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B45">
         <v>201208</v>
       </c>
       <c r="C45" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F45" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B46">
         <v>714</v>
       </c>
       <c r="C46" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F46" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B47">
         <v>171365</v>
       </c>
       <c r="C47" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F47" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B48">
         <v>209439</v>
       </c>
       <c r="C48" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F48" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B49">
         <v>209273</v>
       </c>
       <c r="C49" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F49" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B50">
         <v>226683</v>
       </c>
       <c r="C50" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F50" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B51">
         <v>226684</v>
       </c>
       <c r="C51" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F51" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52">
         <v>226685</v>
       </c>
       <c r="C52" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F52" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53">
         <v>115460</v>
       </c>
       <c r="C53" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F53" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54">
         <v>205494</v>
       </c>
       <c r="C54" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F54" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55">
         <v>226885</v>
       </c>
       <c r="C55" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F55" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56">
         <v>222699</v>
       </c>
       <c r="C56" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F56" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>226996</v>
       </c>
       <c r="C57" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F57" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="58" spans="2:6">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B58">
         <v>227576</v>
       </c>
       <c r="C58" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F58" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="59" spans="2:6">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59">
         <v>203106</v>
       </c>
       <c r="C59" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F59" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60">
         <v>208992</v>
       </c>
       <c r="C60" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F60" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B61">
         <v>226886</v>
       </c>
       <c r="C61" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F61" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B62">
         <v>175782</v>
       </c>
       <c r="C62" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F62" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B63">
         <v>176588</v>
       </c>
       <c r="C63" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F63" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B64">
         <v>175802</v>
       </c>
       <c r="C64" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F64" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="65" spans="2:6">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B65">
         <v>175703</v>
       </c>
       <c r="C65" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F65" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="66" spans="2:6">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B66">
         <v>173738</v>
       </c>
       <c r="C66" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F66" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B67">
         <v>175702</v>
       </c>
       <c r="C67" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F67" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="68" spans="2:6">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B68">
         <v>1090</v>
       </c>
       <c r="C68" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F68" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="69" spans="2:6">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B69">
         <v>115862</v>
       </c>
       <c r="C69" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F69" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="70" spans="2:6">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B70">
         <v>130023</v>
       </c>
       <c r="C70" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F70" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="71" spans="2:6">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B71">
         <v>205779</v>
       </c>
       <c r="C71" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F71" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="72" spans="2:6">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B72">
         <v>160240</v>
       </c>
       <c r="C72" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F72" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="73" spans="2:6">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B73">
         <v>31509</v>
       </c>
       <c r="C73" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F73" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="74" spans="2:6">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B74">
         <v>31510</v>
       </c>
       <c r="C74" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F74" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="75" spans="2:6">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B75">
         <v>3334</v>
       </c>
       <c r="C75" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F75" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="76" spans="2:6">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B76">
         <v>31179</v>
       </c>
       <c r="C76" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F76" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="77" spans="2:6">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B77">
         <v>3946</v>
       </c>
       <c r="C77" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F77" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="78" spans="2:6">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B78">
         <v>3947</v>
       </c>
       <c r="C78" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F78" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="79" spans="2:6">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B79">
         <v>3948</v>
       </c>
       <c r="C79" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F79" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="80" spans="2:6">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B80">
         <v>3949</v>
       </c>
       <c r="C80" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F80" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="81" spans="2:6">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B81">
         <v>3950</v>
       </c>
       <c r="C81" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F81" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="82" spans="2:6">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B82">
         <v>31600</v>
       </c>
       <c r="C82" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F82" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="83" spans="2:6">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B83">
         <v>3951</v>
       </c>
       <c r="C83" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F83" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="84" spans="2:6">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B84">
         <v>160766</v>
       </c>
       <c r="C84" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F84" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="85" spans="2:6">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B85">
         <v>4311</v>
       </c>
       <c r="C85" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F85" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="86" spans="2:6">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B86">
         <v>771</v>
       </c>
       <c r="C86" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F86" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="87" spans="2:6">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B87">
         <v>772</v>
       </c>
       <c r="C87" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F87" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="88" spans="2:6">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B88">
         <v>773</v>
       </c>
       <c r="C88" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F88" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="89" spans="2:6">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B89">
         <v>775</v>
       </c>
       <c r="C89" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F89" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="90" spans="2:6">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B90">
         <v>777</v>
       </c>
       <c r="C90" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F90" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3911,34 +3835,45 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C1" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D1" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="E1" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F1" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="G1" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="H1" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="I1" t="s">
         <v>2</v>
@@ -3950,37 +3885,37 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C1" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D1" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="E1" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="F1" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="G1" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>17</v>
       </c>
@@ -3991,16 +3926,16 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E2" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="H2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>17</v>
       </c>
@@ -4011,16 +3946,16 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="H3" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>17</v>
       </c>
@@ -4031,16 +3966,16 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E4" t="s">
+        <v>249</v>
+      </c>
+      <c r="H4" t="s">
         <v>258</v>
       </c>
-      <c r="E4" t="s">
-        <v>260</v>
-      </c>
-      <c r="H4" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>17</v>
       </c>
@@ -4051,16 +3986,16 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E5" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="H5" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>17</v>
       </c>
@@ -4071,16 +4006,16 @@
         <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E6" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="H6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>17</v>
       </c>
@@ -4091,16 +4026,16 @@
         <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E7" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="H7" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>17</v>
       </c>
@@ -4111,16 +4046,16 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E8" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="H8" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>17</v>
       </c>
@@ -4131,16 +4066,16 @@
         <v>196</v>
       </c>
       <c r="D9" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E9" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="H9" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>17</v>
       </c>
@@ -4151,16 +4086,16 @@
         <v>123</v>
       </c>
       <c r="D10" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E10" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="H10" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>20</v>
       </c>
@@ -4171,16 +4106,16 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E11" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="H11" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>20</v>
       </c>
@@ -4191,16 +4126,16 @@
         <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E12" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="H12" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>20</v>
       </c>
@@ -4211,16 +4146,16 @@
         <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E13" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="H13" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>20</v>
       </c>
@@ -4231,13 +4166,13 @@
         <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E14" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="H14" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -4246,461 +4181,474 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="69.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>29</v>
       </c>
       <c r="B1" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="C1" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="D1" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="E1" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="F1" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="G1" t="s">
         <v>0</v>
       </c>
       <c r="H1" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="I1" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="J1" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="K1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="B2" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="C2" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D2" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="E2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F2" t="s">
+        <v>324</v>
+      </c>
+      <c r="H2" t="s">
+        <v>328</v>
+      </c>
+      <c r="I2" t="s">
         <v>329</v>
       </c>
-      <c r="F2" t="s">
-        <v>335</v>
-      </c>
-      <c r="H2" t="s">
-        <v>339</v>
-      </c>
-      <c r="I2" t="s">
-        <v>340</v>
-      </c>
       <c r="J2" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="K2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="B3" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="C3" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D3" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="E3" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="F3" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="G3">
         <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="I3" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="J3" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="K3" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="B4" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="C4" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D4" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="s">
+        <v>325</v>
+      </c>
+      <c r="H4" t="s">
+        <v>328</v>
+      </c>
+      <c r="I4" t="s">
+        <v>329</v>
+      </c>
+      <c r="J4" t="s">
+        <v>330</v>
+      </c>
+      <c r="K4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>280</v>
+      </c>
+      <c r="B5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" t="s">
+        <v>304</v>
+      </c>
+      <c r="D5" t="s">
+        <v>314</v>
+      </c>
+      <c r="F5" t="s">
+        <v>325</v>
+      </c>
+      <c r="H5" t="s">
+        <v>328</v>
+      </c>
+      <c r="I5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J5" t="s">
+        <v>330</v>
+      </c>
+      <c r="K5" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F6" t="s">
+        <v>326</v>
+      </c>
+      <c r="H6" t="s">
+        <v>328</v>
+      </c>
+      <c r="I6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J6" t="s">
+        <v>330</v>
+      </c>
+      <c r="K6" t="s">
         <v>336</v>
       </c>
-      <c r="H4" t="s">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>282</v>
+      </c>
+      <c r="B7" t="s">
+        <v>295</v>
+      </c>
+      <c r="C7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D7" t="s">
+        <v>314</v>
+      </c>
+      <c r="F7" t="s">
+        <v>324</v>
+      </c>
+      <c r="H7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I7" t="s">
+        <v>328</v>
+      </c>
+      <c r="J7" t="s">
+        <v>330</v>
+      </c>
+      <c r="K7" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>283</v>
+      </c>
+      <c r="B8" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" t="s">
+        <v>314</v>
+      </c>
+      <c r="F8" t="s">
+        <v>326</v>
+      </c>
+      <c r="H8" t="s">
+        <v>328</v>
+      </c>
+      <c r="I8" t="s">
+        <v>328</v>
+      </c>
+      <c r="J8" t="s">
+        <v>330</v>
+      </c>
+      <c r="K8" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>284</v>
+      </c>
+      <c r="B9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" t="s">
+        <v>308</v>
+      </c>
+      <c r="D9" t="s">
+        <v>315</v>
+      </c>
+      <c r="E9" t="s">
+        <v>320</v>
+      </c>
+      <c r="F9" t="s">
+        <v>325</v>
+      </c>
+      <c r="H9" t="s">
+        <v>328</v>
+      </c>
+      <c r="I9" t="s">
+        <v>328</v>
+      </c>
+      <c r="J9" t="s">
+        <v>330</v>
+      </c>
+      <c r="K9" t="s">
         <v>339</v>
       </c>
-      <c r="I4" t="s">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>285</v>
+      </c>
+      <c r="B10" t="s">
+        <v>298</v>
+      </c>
+      <c r="C10" t="s">
+        <v>309</v>
+      </c>
+      <c r="D10" t="s">
+        <v>313</v>
+      </c>
+      <c r="E10" t="s">
+        <v>321</v>
+      </c>
+      <c r="F10" t="s">
+        <v>325</v>
+      </c>
+      <c r="H10" t="s">
+        <v>328</v>
+      </c>
+      <c r="I10" t="s">
+        <v>329</v>
+      </c>
+      <c r="J10" t="s">
+        <v>331</v>
+      </c>
+      <c r="K10" t="s">
         <v>340</v>
       </c>
-      <c r="J4" t="s">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" t="s">
+        <v>299</v>
+      </c>
+      <c r="C11" t="s">
+        <v>310</v>
+      </c>
+      <c r="D11" t="s">
+        <v>314</v>
+      </c>
+      <c r="F11" t="s">
+        <v>325</v>
+      </c>
+      <c r="H11" t="s">
+        <v>329</v>
+      </c>
+      <c r="I11" t="s">
+        <v>329</v>
+      </c>
+      <c r="J11" t="s">
+        <v>330</v>
+      </c>
+      <c r="K11" t="s">
         <v>341</v>
       </c>
-      <c r="K4" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
-        <v>291</v>
-      </c>
-      <c r="B5" t="s">
-        <v>304</v>
-      </c>
-      <c r="C5" t="s">
-        <v>315</v>
-      </c>
-      <c r="D5" t="s">
-        <v>325</v>
-      </c>
-      <c r="F5" t="s">
-        <v>336</v>
-      </c>
-      <c r="H5" t="s">
-        <v>339</v>
-      </c>
-      <c r="I5" t="s">
-        <v>340</v>
-      </c>
-      <c r="J5" t="s">
-        <v>341</v>
-      </c>
-      <c r="K5" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>292</v>
-      </c>
-      <c r="B6" t="s">
-        <v>305</v>
-      </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" t="s">
+        <v>300</v>
+      </c>
+      <c r="C12" t="s">
+        <v>311</v>
+      </c>
+      <c r="D12" t="s">
         <v>316</v>
       </c>
-      <c r="D6" t="s">
-        <v>325</v>
-      </c>
-      <c r="F6" t="s">
-        <v>337</v>
-      </c>
-      <c r="H6" t="s">
-        <v>339</v>
-      </c>
-      <c r="I6" t="s">
-        <v>340</v>
-      </c>
-      <c r="J6" t="s">
-        <v>341</v>
-      </c>
-      <c r="K6" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" t="s">
-        <v>293</v>
-      </c>
-      <c r="B7" t="s">
-        <v>306</v>
-      </c>
-      <c r="C7" t="s">
-        <v>317</v>
-      </c>
-      <c r="D7" t="s">
-        <v>325</v>
-      </c>
-      <c r="F7" t="s">
-        <v>335</v>
-      </c>
-      <c r="H7" t="s">
-        <v>339</v>
-      </c>
-      <c r="I7" t="s">
-        <v>339</v>
-      </c>
-      <c r="J7" t="s">
-        <v>341</v>
-      </c>
-      <c r="K7" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" t="s">
-        <v>294</v>
-      </c>
-      <c r="B8" t="s">
-        <v>307</v>
-      </c>
-      <c r="C8" t="s">
-        <v>318</v>
-      </c>
-      <c r="D8" t="s">
-        <v>325</v>
-      </c>
-      <c r="F8" t="s">
-        <v>337</v>
-      </c>
-      <c r="H8" t="s">
-        <v>339</v>
-      </c>
-      <c r="I8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J8" t="s">
-        <v>341</v>
-      </c>
-      <c r="K8" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" t="s">
-        <v>295</v>
-      </c>
-      <c r="B9" t="s">
-        <v>308</v>
-      </c>
-      <c r="C9" t="s">
-        <v>319</v>
-      </c>
-      <c r="D9" t="s">
-        <v>326</v>
-      </c>
-      <c r="E9" t="s">
-        <v>331</v>
-      </c>
-      <c r="F9" t="s">
-        <v>336</v>
-      </c>
-      <c r="H9" t="s">
-        <v>339</v>
-      </c>
-      <c r="I9" t="s">
-        <v>339</v>
-      </c>
-      <c r="J9" t="s">
-        <v>341</v>
-      </c>
-      <c r="K9" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" t="s">
-        <v>296</v>
-      </c>
-      <c r="B10" t="s">
-        <v>309</v>
-      </c>
-      <c r="C10" t="s">
-        <v>320</v>
-      </c>
-      <c r="D10" t="s">
-        <v>324</v>
-      </c>
-      <c r="E10" t="s">
-        <v>332</v>
-      </c>
-      <c r="F10" t="s">
-        <v>336</v>
-      </c>
-      <c r="H10" t="s">
-        <v>339</v>
-      </c>
-      <c r="I10" t="s">
-        <v>340</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="E12" t="s">
+        <v>322</v>
+      </c>
+      <c r="F12" t="s">
+        <v>327</v>
+      </c>
+      <c r="H12" t="s">
+        <v>329</v>
+      </c>
+      <c r="I12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J12" t="s">
+        <v>330</v>
+      </c>
+      <c r="K12" t="s">
         <v>342</v>
       </c>
-      <c r="K10" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" t="s">
-        <v>297</v>
-      </c>
-      <c r="B11" t="s">
-        <v>310</v>
-      </c>
-      <c r="C11" t="s">
-        <v>321</v>
-      </c>
-      <c r="D11" t="s">
-        <v>325</v>
-      </c>
-      <c r="F11" t="s">
-        <v>336</v>
-      </c>
-      <c r="H11" t="s">
-        <v>340</v>
-      </c>
-      <c r="I11" t="s">
-        <v>340</v>
-      </c>
-      <c r="J11" t="s">
-        <v>341</v>
-      </c>
-      <c r="K11" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
-      <c r="A12" t="s">
-        <v>298</v>
-      </c>
-      <c r="B12" t="s">
-        <v>311</v>
-      </c>
-      <c r="C12" t="s">
-        <v>322</v>
-      </c>
-      <c r="D12" t="s">
-        <v>327</v>
-      </c>
-      <c r="E12" t="s">
-        <v>333</v>
-      </c>
-      <c r="F12" t="s">
-        <v>338</v>
-      </c>
-      <c r="H12" t="s">
-        <v>340</v>
-      </c>
-      <c r="I12" t="s">
-        <v>340</v>
-      </c>
-      <c r="J12" t="s">
-        <v>341</v>
-      </c>
-      <c r="K12" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="B13" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
       </c>
       <c r="D13" t="s">
+        <v>317</v>
+      </c>
+      <c r="E13" t="s">
+        <v>323</v>
+      </c>
+      <c r="F13" t="s">
+        <v>327</v>
+      </c>
+      <c r="H13" t="s">
+        <v>329</v>
+      </c>
+      <c r="I13" t="s">
+        <v>329</v>
+      </c>
+      <c r="J13" t="s">
+        <v>330</v>
+      </c>
+      <c r="K13" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" t="s">
+        <v>302</v>
+      </c>
+      <c r="F14" t="s">
+        <v>326</v>
+      </c>
+      <c r="H14" t="s">
         <v>328</v>
       </c>
-      <c r="E13" t="s">
-        <v>334</v>
-      </c>
-      <c r="F13" t="s">
-        <v>338</v>
-      </c>
-      <c r="H13" t="s">
-        <v>340</v>
-      </c>
-      <c r="I13" t="s">
-        <v>340</v>
-      </c>
-      <c r="J13" t="s">
-        <v>341</v>
-      </c>
-      <c r="K13" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" t="s">
-        <v>300</v>
-      </c>
-      <c r="B14" t="s">
-        <v>313</v>
-      </c>
-      <c r="F14" t="s">
-        <v>337</v>
-      </c>
-      <c r="H14" t="s">
-        <v>339</v>
-      </c>
       <c r="I14" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="J14" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="K14" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="B15" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="F15" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="H15" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="I15" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="J15" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="K15" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -4709,129 +4657,134 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="B1" t="s">
         <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="B3">
         <v>-0.5</v>
       </c>
       <c r="C3" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="B4">
         <v>0.01</v>
       </c>
       <c r="C4" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="B5">
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B6" t="s">
+        <v>357</v>
+      </c>
+      <c r="C6" t="s">
         <v>362</v>
       </c>
-      <c r="B6" t="s">
-        <v>368</v>
-      </c>
-      <c r="C6" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="B7">
         <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="B8">
         <v>0.25</v>
       </c>
       <c r="C8" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="B9">
         <v>0.4</v>
       </c>
       <c r="C9" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="B10">
         <v>0.1</v>
       </c>
       <c r="C10" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="B11">
         <v>0.95</v>
       </c>
       <c r="C11" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>